<commit_message>
Fixes from the M9 audit: export paths, map merge guard, password edge cases
get_data_from_view's timestamped CSV is read from Workbench's output;
printed export paths resolve against the Workbench folder. Merging a CSV
ID map asks first and refuses a map into itself; config paths with commas
are refused. password: with no value counts as set; a credentials file
plus ISLANDORA_WORKBENCH_PASSWORD is refused with the reason; ~\ and
USERPROFILE on Windows; empty secrets are ignored. Spreadsheet times and
durations convert correctly. Profile replace re-reads the active profile.
Quoted-ID warning skips empty strings.
</commit_message>
<xml_diff>
--- a/crates/workbench-integration/tests/fixtures/items.xlsx
+++ b/crates/workbench-integration/tests/fixtures/items.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="Notes" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Items" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Times" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,9 +18,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="166" formatCode="[hh]:mm:ss"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -50,10 +52,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="21" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -489,4 +493,38 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>at</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>took</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="n">
+        <v>0.6041666666666666</v>
+      </c>
+      <c r="B2" s="4" t="n">
+        <v>1.086805555555556</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>